<commit_message>
changes have been done in industry and transport
</commit_message>
<xml_diff>
--- a/transport/trans_config.xlsx
+++ b/transport/trans_config.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://fraunhofer-my.sharepoint.com/personal/rakesh_etikala_narendar_iee_fraunhofer_de/Documents/Desktop/sectoral-energy-demands/transport/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="205" documentId="11_23F921EDAE034F2B492C4C492D40CC9F4213A6C0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3458ECFF-A4F2-48C7-972E-731BE5BA7BAD}"/>
+  <xr:revisionPtr revIDLastSave="213" documentId="11_23F921EDAE034F2B492C4C492D40CC9F4213A6C0" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{91591F53-433F-41E3-9B2F-D670405760AB}"/>
   <bookViews>
-    <workbookView xWindow="19910" yWindow="1770" windowWidth="18450" windowHeight="15580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7380" yWindow="3810" windowWidth="30760" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -904,8 +904,10 @@
     <col min="1" max="1" width="15.36328125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="45.6328125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.7265625" customWidth="1"/>
-    <col min="27" max="27" width="11" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="11.08984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="26" width="0" hidden="1" customWidth="1"/>
+    <col min="27" max="27" width="11" hidden="1" customWidth="1"/>
+    <col min="28" max="28" width="11.08984375" hidden="1" customWidth="1"/>
+    <col min="29" max="30" width="0" hidden="1" customWidth="1"/>
     <col min="35" max="35" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="37" max="37" width="9.54296875" bestFit="1" customWidth="1"/>
     <col min="38" max="38" width="21.08984375" bestFit="1" customWidth="1"/>
@@ -52256,7 +52258,7 @@
         <v>0.88</v>
       </c>
     </row>
-    <row r="545" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="545" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A545" t="s">
         <v>73</v>
       </c>
@@ -52273,7 +52275,7 @@
         <v>0.95</v>
       </c>
     </row>
-    <row r="546" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="546" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A546" t="s">
         <v>73</v>
       </c>
@@ -52290,7 +52292,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="547" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="547" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A547" t="s">
         <v>73</v>
       </c>
@@ -52306,8 +52308,11 @@
       <c r="E547">
         <v>7.0000000000000007E-2</v>
       </c>
-    </row>
-    <row r="548" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="AE547">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A548" t="s">
         <v>73</v>
       </c>
@@ -52324,7 +52329,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="549" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="549" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A549" t="s">
         <v>73</v>
       </c>
@@ -52341,7 +52346,7 @@
         <v>0.06</v>
       </c>
     </row>
-    <row r="550" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="550" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A550" t="s">
         <v>73</v>
       </c>
@@ -52358,7 +52363,7 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="551" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="551" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A551" t="s">
         <v>73</v>
       </c>
@@ -52375,7 +52380,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="552" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="552" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A552" t="s">
         <v>73</v>
       </c>
@@ -52392,7 +52397,7 @@
         <v>0.75</v>
       </c>
     </row>
-    <row r="553" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="553" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A553" t="s">
         <v>73</v>
       </c>
@@ -52408,8 +52413,11 @@
       <c r="E553">
         <v>0.92</v>
       </c>
-    </row>
-    <row r="554" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="AE553">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="554" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A554" t="s">
         <v>73</v>
       </c>
@@ -52426,7 +52434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="555" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="555" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A555" t="s">
         <v>73</v>
       </c>
@@ -52443,7 +52451,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="556" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="556" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A556" t="s">
         <v>73</v>
       </c>
@@ -52460,7 +52468,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="557" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="557" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A557" t="s">
         <v>73</v>
       </c>
@@ -52477,7 +52485,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="558" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="558" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A558" t="s">
         <v>73</v>
       </c>
@@ -52494,7 +52502,7 @@
         <v>0.09</v>
       </c>
     </row>
-    <row r="559" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="559" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A559" t="s">
         <v>73</v>
       </c>
@@ -52510,8 +52518,11 @@
       <c r="E559">
         <v>0.01</v>
       </c>
-    </row>
-    <row r="560" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="AE559">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="560" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A560" t="s">
         <v>73</v>
       </c>
@@ -52800,7 +52811,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="577" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="577" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A577" t="s">
         <v>73</v>
       </c>
@@ -52817,7 +52828,7 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="578" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="578" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A578" t="s">
         <v>73</v>
       </c>
@@ -52834,7 +52845,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="579" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="579" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A579" t="s">
         <v>73</v>
       </c>
@@ -52851,7 +52862,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="580" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="580" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A580" t="s">
         <v>73</v>
       </c>
@@ -52868,7 +52879,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="581" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="581" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A581" t="s">
         <v>73</v>
       </c>
@@ -52885,7 +52896,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="582" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="582" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A582" t="s">
         <v>73</v>
       </c>
@@ -52902,7 +52913,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="583" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="583" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A583" t="s">
         <v>73</v>
       </c>
@@ -52919,7 +52930,7 @@
         <v>0.05</v>
       </c>
     </row>
-    <row r="584" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="584" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A584" t="s">
         <v>73</v>
       </c>
@@ -52936,7 +52947,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="585" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="585" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A585" t="s">
         <v>73</v>
       </c>
@@ -52953,7 +52964,7 @@
         <v>0.65</v>
       </c>
     </row>
-    <row r="586" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="586" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A586" t="s">
         <v>73</v>
       </c>
@@ -52970,7 +52981,7 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="587" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="587" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A587" t="s">
         <v>73</v>
       </c>
@@ -52987,7 +52998,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="588" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="588" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A588" t="s">
         <v>73</v>
       </c>
@@ -53004,7 +53015,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="589" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="589" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A589" t="s">
         <v>73</v>
       </c>
@@ -53020,8 +53031,11 @@
       <c r="E589">
         <v>0.5</v>
       </c>
-    </row>
-    <row r="590" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="AE589">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="590" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A590" t="s">
         <v>73</v>
       </c>
@@ -53038,7 +53052,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="591" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="591" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A591" t="s">
         <v>73</v>
       </c>
@@ -53055,7 +53069,7 @@
         <v>0.25</v>
       </c>
     </row>
-    <row r="592" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="592" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A592" t="s">
         <v>73</v>
       </c>
@@ -53072,7 +53086,7 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="593" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="593" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A593" t="s">
         <v>73</v>
       </c>
@@ -53089,7 +53103,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="594" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="594" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A594" t="s">
         <v>73</v>
       </c>
@@ -53106,7 +53120,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="595" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="595" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A595" t="s">
         <v>73</v>
       </c>
@@ -53123,7 +53137,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="596" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="596" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A596" t="s">
         <v>73</v>
       </c>
@@ -53140,7 +53154,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="597" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="597" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A597" t="s">
         <v>73</v>
       </c>
@@ -53157,7 +53171,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="598" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="598" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A598" t="s">
         <v>73</v>
       </c>
@@ -53174,7 +53188,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="599" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="599" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A599" t="s">
         <v>73</v>
       </c>
@@ -53191,7 +53205,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="600" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="600" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A600" t="s">
         <v>73</v>
       </c>
@@ -53208,7 +53222,7 @@
         <v>0.35</v>
       </c>
     </row>
-    <row r="601" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="601" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A601" t="s">
         <v>73</v>
       </c>
@@ -53224,8 +53238,11 @@
       <c r="E601">
         <v>0.38</v>
       </c>
-    </row>
-    <row r="602" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="AE601">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="602" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A602" t="s">
         <v>73</v>
       </c>
@@ -53242,7 +53259,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="603" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="603" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A603" t="s">
         <v>73</v>
       </c>
@@ -53259,7 +53276,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="604" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="604" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A604" t="s">
         <v>73</v>
       </c>
@@ -53276,7 +53293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="605" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="605" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A605" t="s">
         <v>73</v>
       </c>
@@ -53293,7 +53310,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="606" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="606" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A606" t="s">
         <v>73</v>
       </c>
@@ -53310,7 +53327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="607" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="607" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A607" t="s">
         <v>73</v>
       </c>
@@ -53327,7 +53344,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="608" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="608" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A608" t="s">
         <v>73</v>
       </c>
@@ -53344,7 +53361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="609" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="609" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A609" t="s">
         <v>73</v>
       </c>
@@ -53361,7 +53378,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="610" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="610" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A610" t="s">
         <v>73</v>
       </c>
@@ -53378,7 +53395,7 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="611" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="611" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A611" t="s">
         <v>73</v>
       </c>
@@ -53395,7 +53412,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="612" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="612" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A612" t="s">
         <v>73</v>
       </c>
@@ -53412,7 +53429,7 @@
         <v>0.15</v>
       </c>
     </row>
-    <row r="613" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="613" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A613" t="s">
         <v>73</v>
       </c>
@@ -53428,8 +53445,11 @@
       <c r="E613">
         <v>0.02</v>
       </c>
-    </row>
-    <row r="614" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="AE613">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="614" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A614" t="s">
         <v>73</v>
       </c>
@@ -53446,7 +53466,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="615" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="615" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A615" t="s">
         <v>73</v>
       </c>
@@ -53463,7 +53483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="616" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="616" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A616" t="s">
         <v>73</v>
       </c>
@@ -53480,7 +53500,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="617" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="617" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A617" t="s">
         <v>73</v>
       </c>
@@ -53497,7 +53517,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="618" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="618" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A618" t="s">
         <v>73</v>
       </c>
@@ -53514,7 +53534,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="619" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="619" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A619" t="s">
         <v>73</v>
       </c>
@@ -53531,7 +53551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="620" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="620" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A620" t="s">
         <v>73</v>
       </c>
@@ -53548,7 +53568,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="621" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="621" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A621" t="s">
         <v>73</v>
       </c>
@@ -53565,7 +53585,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="622" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="622" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A622" t="s">
         <v>73</v>
       </c>
@@ -53582,7 +53602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="623" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="623" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A623" t="s">
         <v>73</v>
       </c>
@@ -53599,7 +53619,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="624" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="624" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A624" t="s">
         <v>73</v>
       </c>
@@ -53888,7 +53908,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="641" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="641" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A641" t="s">
         <v>73</v>
       </c>
@@ -53905,7 +53925,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="642" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="642" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A642" t="s">
         <v>73</v>
       </c>
@@ -53922,7 +53942,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="643" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="643" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A643" t="s">
         <v>73</v>
       </c>
@@ -53939,7 +53959,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="644" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="644" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A644" t="s">
         <v>73</v>
       </c>
@@ -53956,7 +53976,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="645" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="645" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A645" t="s">
         <v>73</v>
       </c>
@@ -53973,7 +53993,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="646" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="646" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A646" t="s">
         <v>73</v>
       </c>
@@ -53990,7 +54010,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="647" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="647" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A647" t="s">
         <v>73</v>
       </c>
@@ -54007,7 +54027,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="648" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="648" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A648" t="s">
         <v>73</v>
       </c>
@@ -54024,7 +54044,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="649" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="649" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A649" t="s">
         <v>73</v>
       </c>
@@ -54041,7 +54061,7 @@
         <v>0.45</v>
       </c>
     </row>
-    <row r="650" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="650" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A650" t="s">
         <v>73</v>
       </c>
@@ -54058,7 +54078,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="651" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="651" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A651" t="s">
         <v>73</v>
       </c>
@@ -54075,7 +54095,7 @@
         <v>0.02</v>
       </c>
     </row>
-    <row r="652" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="652" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A652" t="s">
         <v>73</v>
       </c>
@@ -54092,7 +54112,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="653" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="653" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A653" t="s">
         <v>73</v>
       </c>
@@ -54109,7 +54129,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="654" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="654" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A654" t="s">
         <v>73</v>
       </c>
@@ -54126,7 +54146,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="655" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="655" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A655" t="s">
         <v>73</v>
       </c>
@@ -54142,8 +54162,11 @@
       <c r="E655">
         <v>0.25</v>
       </c>
-    </row>
-    <row r="656" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="AE655">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="656" spans="1:31" x14ac:dyDescent="0.35">
       <c r="A656" t="s">
         <v>73</v>
       </c>

</xml_diff>